<commit_message>
j1,j2,,j3 mais pas tout
</commit_message>
<xml_diff>
--- a/todoJ1.xlsx
+++ b/todoJ1.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="36">
   <si>
     <t xml:space="preserve">ORDRE</t>
   </si>
@@ -46,10 +46,16 @@
     <t xml:space="preserve">Back Office</t>
   </si>
   <si>
-    <t xml:space="preserve">en cours </t>
+    <t xml:space="preserve">termine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">j1</t>
   </si>
   <si>
     <t xml:space="preserve">créer une page avec un bouton pour réinitialiser les données </t>
+  </si>
+  <si>
+    <t xml:space="preserve">termine </t>
   </si>
   <si>
     <t xml:space="preserve">créer la page pour importer les 4 fichiers </t>
@@ -79,21 +85,68 @@
   </si>
   <si>
     <t xml:space="preserve">Ajout état de “mes commandes” </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mise a jour des etats de commande </t>
+  </si>
+  <si>
+    <t xml:space="preserve">j2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ajout de tableau de bord du. nb de commande et montant par jour et    Total général </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ajout de la page d’inscription des utilisateurs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mise a jour sur la page d’acceuil le choix d’utilisateur pour se connecter a la boutique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ajout d’un utilisateur Anonyme</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ajout de marque sur les produits ( NEW  et HOT)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">implémenter une recherche multicritère par produit ,nom,categorie,intervalle de prix</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rajouter une page qui permet d’ajouter en stock les produits </t>
+  </si>
+  <si>
+    <t xml:space="preserve">en cours</t>
+  </si>
+  <si>
+    <t xml:space="preserve">j3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Afficher la quantité en stock disponible sur la fiche produit </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vérifier les erreurs suivants dans l’import : Nom de colonne non conforme </t>
+  </si>
+  <si>
+    <t xml:space="preserve">format de date différente de DD/MM/YYYY </t>
+  </si>
+  <si>
+    <t xml:space="preserve">montant positif </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.00\ %"/>
+    <numFmt numFmtId="166" formatCode="#,##0.00"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -130,6 +183,13 @@
       <sz val="10"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -179,40 +239,64 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -339,194 +423,443 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="53.97"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24.34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20.03"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="21.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="25.32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="25.74"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="20.03"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="26.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="23.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="70.81"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="24.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="20.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="21.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="25.32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="25.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="20.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="26.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="23.65"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1"/>
-      <c r="J1" s="3"/>
+      <c r="G1" s="2"/>
+      <c r="J1" s="4"/>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="n">
+      <c r="A2" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="F2" s="6" t="n">
+      <c r="C2" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2" s="7" t="n">
         <v>0.2</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="n">
+      <c r="A3" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="F3" s="6" t="n">
+      <c r="F3" s="7" t="n">
         <v>0.5</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="n">
+      <c r="A4" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F6" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F7" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F9" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E10" s="5"/>
+      <c r="F10" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="4" t="s">
+      <c r="B11" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="10" t="n">
         <v>11</v>
       </c>
-      <c r="F4" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="5" t="s">
+      <c r="B12" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="10" t="n">
         <v>12</v>
       </c>
-      <c r="C5" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="F5" s="6" t="n">
-        <v>0.8</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="5" t="s">
+      <c r="B13" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="10" t="n">
         <v>13</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="B14" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="10" t="n">
         <v>14</v>
       </c>
-      <c r="D6" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F6" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="5" t="s">
+      <c r="B15" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="10" t="n">
         <v>15</v>
       </c>
-      <c r="C7" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F7" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F8" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="8" t="s">
+      <c r="B16" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="10" t="n">
         <v>17</v>
       </c>
-      <c r="C9" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F9" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="5" t="s">
+      <c r="B18" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="10" t="n">
         <v>18</v>
       </c>
-      <c r="C10" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F10" s="7" t="n">
-        <v>0</v>
-      </c>
+      <c r="B19" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="10" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D24" s="5"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>